<commit_message>
feat(m9): toi uu layout Partnership, cap nhat Dining City T7-T8 va bieu do co cau doi tac
</commit_message>
<xml_diff>
--- a/data_input/01_master.xlsx
+++ b/data_input/01_master.xlsx
@@ -16,14 +16,16 @@
     <sheet name="budget_channel" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="budget_store" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="partners" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="partner_camp" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="pre_analytics" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="crm_target" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="system_tools" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="system_dashboards" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="system_caches" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="_stats" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="partner_plan" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="pre_analytics" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="crm_target" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="system_tools" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="system_dashboards" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="system_caches" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="_stats" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="partner_plan" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="partner_program" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="partner_agg" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="partner_voucher" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -814,142 +816,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>code</t>
-        </is>
-      </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="C1" s="5" t="inlineStr">
-        <is>
-          <t>cid</t>
-        </is>
-      </c>
-      <c r="D1" s="5" t="inlineStr">
-        <is>
-          <t>mech</t>
-        </is>
-      </c>
-      <c r="E1" s="5" t="inlineStr">
-        <is>
-          <t>rate</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>P01</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Noire - Techcombank Reward × OneU</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>337795</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Chiết khấu %</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
-        <v>0.15</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>P02</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Hoa hồng</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>P03</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>GRAB DINE OUT</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Chiết khấu %</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>P04</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Chiết khấu %</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>0.15</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>P05</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Giảm 10% cho thẻ Shinhan Bank hoặc Shinhan Finance</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Chiết khấu %</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>0.1</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1584,7 +1450,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1795,7 +1661,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1945,7 +1811,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2146,7 +2012,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2234,7 +2100,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2407,19 +2273,643 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>scenario</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>issued</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>use_rate</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>aov</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>rev</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>cost</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>gp</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Cơ sở</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F2" t="n">
+        <v>325151</v>
+      </c>
+      <c r="G2" t="n">
+        <v>81287750</v>
+      </c>
+      <c r="H2" t="n">
+        <v>12193162.5</v>
+      </c>
+      <c r="I2" t="n">
+        <v>43082507.5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Cơ sở</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F3" t="n">
+        <v>325151</v>
+      </c>
+      <c r="G3" t="n">
+        <v>81287750</v>
+      </c>
+      <c r="H3" t="n">
+        <v>12193162.5</v>
+      </c>
+      <c r="I3" t="n">
+        <v>43082507.5</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Cơ sở</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F4" t="n">
+        <v>325151</v>
+      </c>
+      <c r="G4" t="n">
+        <v>81287750</v>
+      </c>
+      <c r="H4" t="n">
+        <v>12193162.5</v>
+      </c>
+      <c r="I4" t="n">
+        <v>43082507.5</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Cơ sở</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F5" t="n">
+        <v>325151</v>
+      </c>
+      <c r="G5" t="n">
+        <v>81287750</v>
+      </c>
+      <c r="H5" t="n">
+        <v>12193162.5</v>
+      </c>
+      <c r="I5" t="n">
+        <v>43082507.5</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-11</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Cơ sở</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F6" t="n">
+        <v>325151</v>
+      </c>
+      <c r="G6" t="n">
+        <v>81287750</v>
+      </c>
+      <c r="H6" t="n">
+        <v>12193162.5</v>
+      </c>
+      <c r="I6" t="n">
+        <v>43082507.5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-12</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Cơ sở</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F7" t="n">
+        <v>325151</v>
+      </c>
+      <c r="G7" t="n">
+        <v>81287750</v>
+      </c>
+      <c r="H7" t="n">
+        <v>12193162.5</v>
+      </c>
+      <c r="I7" t="n">
+        <v>43082507.5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>P02</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Cơ sở</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>2902750</v>
+      </c>
+      <c r="G8" t="n">
+        <v>14513750</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>P02</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Cơ sở</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>2902750</v>
+      </c>
+      <c r="G9" t="n">
+        <v>17416500</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>P02</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Cơ sở</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>2902750</v>
+      </c>
+      <c r="G10" t="n">
+        <v>20319250</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>P02</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Cơ sở</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
+        <v>2902750</v>
+      </c>
+      <c r="G11" t="n">
+        <v>20319250</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-11</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>P02</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Cơ sở</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>2902750</v>
+      </c>
+      <c r="G12" t="n">
+        <v>23222000</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-12</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>P02</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Cơ sở</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="n">
+        <v>2902750</v>
+      </c>
+      <c r="G13" t="n">
+        <v>26124750</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>P04</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Cơ sở</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>689989</v>
+      </c>
+      <c r="G14" t="n">
+        <v>13799780</v>
+      </c>
+      <c r="H14" t="n">
+        <v>2069967</v>
+      </c>
+      <c r="I14" t="n">
+        <v>7313883.333</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>P04</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Cơ sở</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>689989</v>
+      </c>
+      <c r="G15" t="n">
+        <v>13799780</v>
+      </c>
+      <c r="H15" t="n">
+        <v>2069967</v>
+      </c>
+      <c r="I15" t="n">
+        <v>7313883.333</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>P04</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Cơ sở</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>689989</v>
+      </c>
+      <c r="G16" t="n">
+        <v>13799780</v>
+      </c>
+      <c r="H16" t="n">
+        <v>2069967</v>
+      </c>
+      <c r="I16" t="n">
+        <v>7313883.333</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>P04</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Cơ sở</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>689989</v>
+      </c>
+      <c r="G17" t="n">
+        <v>13799780</v>
+      </c>
+      <c r="H17" t="n">
+        <v>2069967</v>
+      </c>
+      <c r="I17" t="n">
+        <v>7313883.333</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-11</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>P04</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Cơ sở</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="n">
+        <v>689989</v>
+      </c>
+      <c r="G18" t="n">
+        <v>13799780</v>
+      </c>
+      <c r="H18" t="n">
+        <v>2069967</v>
+      </c>
+      <c r="I18" t="n">
+        <v>7313883.333</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-12</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>P04</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Cơ sở</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" t="n">
+        <v>689989</v>
+      </c>
+      <c r="G19" t="n">
+        <v>13799780</v>
+      </c>
+      <c r="H19" t="n">
+        <v>2069967</v>
+      </c>
+      <c r="I19" t="n">
+        <v>7313883.333</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>month</t>
+          <t>prog</t>
         </is>
       </c>
       <c r="B1" s="5" t="inlineStr">
@@ -2429,44 +2919,79 @@
       </c>
       <c r="C1" s="5" t="inlineStr">
         <is>
-          <t>scenario</t>
+          <t>name</t>
         </is>
       </c>
       <c r="D1" s="5" t="inlineStr">
         <is>
-          <t>issued</t>
+          <t>brand</t>
         </is>
       </c>
       <c r="E1" s="5" t="inlineStr">
         <is>
-          <t>use_rate</t>
+          <t>mech</t>
         </is>
       </c>
       <c r="F1" s="5" t="inlineStr">
         <is>
-          <t>aov</t>
+          <t>offer</t>
         </is>
       </c>
       <c r="G1" s="5" t="inlineStr">
         <is>
-          <t>cost</t>
+          <t>rate</t>
         </is>
       </c>
       <c r="H1" s="5" t="inlineStr">
         <is>
-          <t>rev</t>
+          <t>cap</t>
         </is>
       </c>
       <c r="I1" s="5" t="inlineStr">
         <is>
-          <t>gp</t>
+          <t>min_bill</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>condition</t>
+        </is>
+      </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+      <c r="L1" s="5" t="inlineStr">
+        <is>
+          <t>end</t>
+        </is>
+      </c>
+      <c r="M1" s="5" t="inlineStr">
+        <is>
+          <t>codes</t>
+        </is>
+      </c>
+      <c r="N1" s="5" t="inlineStr">
+        <is>
+          <t>cid</t>
+        </is>
+      </c>
+      <c r="O1" s="5" t="inlineStr">
+        <is>
+          <t>pos_name</t>
+        </is>
+      </c>
+      <c r="P1" s="5" t="inlineStr">
+        <is>
+          <t>note</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-07</t>
+          <t>P01-NCB</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2476,32 +3001,66 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Cơ sở</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>1000</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="F2" t="n">
-        <v>325151</v>
+          <t>Noire - Techcombank Reward × OneU</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>NCB</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Mã e-voucher</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Giảm 15% hoá đơn, tối đa 100.000đ, hoá đơn từ 300.000đ</t>
+        </is>
       </c>
       <c r="G2" t="n">
-        <v>12193162.5</v>
+        <v>0.15</v>
       </c>
       <c r="H2" t="n">
-        <v>81287750</v>
+        <v>100000</v>
       </c>
       <c r="I2" t="n">
-        <v>43082507.5</v>
+        <v>300000</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="M2" t="n">
+        <v>3000</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>337795</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Noire - Techcombank Reward × OneU</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Log eVoucher: mã TC…, phát 1 lô 21/07</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>P01-NDC</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -2511,32 +3070,60 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Cơ sở</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>1000</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="F3" t="n">
-        <v>325151</v>
+          <t>Dining - Techcombank Reward × OneU</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>NDC</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Mã e-voucher</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Giảm 200.000đ / hoá đơn</t>
+        </is>
       </c>
       <c r="G3" t="n">
-        <v>12193162.5</v>
-      </c>
-      <c r="H3" t="n">
-        <v>81287750</v>
-      </c>
-      <c r="I3" t="n">
-        <v>43082507.5</v>
+        <v>200000</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="M3" t="n">
+        <v>1500</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>344574</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Dining - Techcombank Reward × OneU</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Mức giảm lấy từ log eVoucher (mọi lượt dùng giảm đúng 200.000đ) — bổ sung HĐ tối thiểu</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>P01-NJFB</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -2546,479 +3133,1278 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Cơ sở</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>1000</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="F4" t="n">
-        <v>325151</v>
+          <t>JFB - Techcombank Reward × OneU</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>NJFB</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Mã e-voucher</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Giảm 400.000đ / hoá đơn</t>
+        </is>
       </c>
       <c r="G4" t="n">
-        <v>12193162.5</v>
-      </c>
-      <c r="H4" t="n">
-        <v>81287750</v>
-      </c>
-      <c r="I4" t="n">
-        <v>43082507.5</v>
+        <v>400000</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="M4" t="n">
+        <v>1500</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>344575</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>JFB - Techcombank Reward × OneU</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Mức giảm lấy từ log eVoucher (mọi lượt dùng giảm đúng 400.000đ) — bổ sung HĐ tối thiểu</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10</t>
+          <t>P04-NDC</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>P01</t>
+          <t>P04</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Cơ sở</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>1000</v>
-      </c>
-      <c r="E5" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="F5" t="n">
-        <v>325151</v>
+          <t>HDBank Priority</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>NDC</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Giảm % hoá đơn</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Giảm 15% tổng hoá đơn cho khách HDBank Priority</t>
+        </is>
       </c>
       <c r="G5" t="n">
-        <v>12193162.5</v>
-      </c>
-      <c r="H5" t="n">
-        <v>81287750</v>
-      </c>
-      <c r="I5" t="n">
-        <v>43082507.5</v>
+        <v>0.15</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-11</t>
+          <t>P05-ALL</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>P01</t>
+          <t>P05</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Cơ sở</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>1000</v>
-      </c>
-      <c r="E6" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="F6" t="n">
-        <v>325151</v>
+          <t>Giảm 10% thẻ Shinhan</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>TẤT CẢ</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Quẹt thẻ tại quầy</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Giảm 10% hoá đơn khi thanh toán bằng thẻ Shinhan Bank / Shinhan Finance</t>
+        </is>
       </c>
       <c r="G6" t="n">
-        <v>12193162.5</v>
-      </c>
-      <c r="H6" t="n">
-        <v>81287750</v>
-      </c>
-      <c r="I6" t="n">
-        <v>43082507.5</v>
+        <v>0.1</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Giảm 10% cho thẻ Shinhan Bank hoặc Shinhan Finance</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-12</t>
+          <t>P03-1</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>P01</t>
+          <t>P03</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Cơ sở</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>1000</v>
-      </c>
-      <c r="E7" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="F7" t="n">
-        <v>325151</v>
+          <t>Grab Dine Out — giảm ngay</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>NDC, NJFB</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Giảm % hoá đơn</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Giảm ngay 20% cho khách mới · 15% cho khách đã dùng Grab Dine Out</t>
+        </is>
       </c>
       <c r="G7" t="n">
-        <v>12193162.5</v>
-      </c>
-      <c r="H7" t="n">
-        <v>81287750</v>
-      </c>
-      <c r="I7" t="n">
-        <v>43082507.5</v>
+        <v>0.2</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>GRAB DINE OUT</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>NOIRE fund</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-07</t>
+          <t>P03-2</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>P02</t>
+          <t>P03</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Cơ sở</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" t="n">
-        <v>2902750</v>
-      </c>
-      <c r="H8" t="n">
-        <v>14513750</v>
+          <t>Grab Dine Out — voucher bán trước</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>NDC, NJFB</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Voucher bán trước</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Voucher 500.000đ mở bán 375.000đ trên Grab</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>125000</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>NOIRE fund</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>P02-1</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>P02</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Dining City — đặt bàn trước</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>NDC, NJFB</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Đặt bàn trước</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Khách đặt bàn qua Dining City</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Hoa hồng 18.000đ/booking</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>brand</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>store</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>bookings</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>cancels</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>guests</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>bills</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>net</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>disc_noire</t>
+        </is>
+      </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>disc_platform</t>
+        </is>
+      </c>
+      <c r="L1" s="5" t="inlineStr">
+        <is>
+          <t>commission</t>
+        </is>
+      </c>
+      <c r="M1" s="5" t="inlineStr">
+        <is>
+          <t>fee_other</t>
+        </is>
+      </c>
+      <c r="N1" s="5" t="inlineStr">
+        <is>
+          <t>method</t>
+        </is>
+      </c>
+      <c r="O1" s="5" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>NDC</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>P02</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I2" t="n">
+        <v>3789933</v>
+      </c>
+      <c r="L2" t="n">
+        <v>36000</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>18.000đ/booking</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>2 booking × 18.000đ = 36.000đ</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
           <t>2026-08</t>
         </is>
       </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>NDC</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>P02</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>20</v>
+      </c>
+      <c r="F3" t="n">
+        <v>7</v>
+      </c>
+      <c r="G3" t="n">
+        <v>32</v>
+      </c>
+      <c r="H3" t="n">
+        <v>13</v>
+      </c>
+      <c r="I3" t="n">
+        <v>8423714</v>
+      </c>
+      <c r="L3" t="n">
+        <v>360000</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>18.000đ/booking</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Báo cáo Promotion-AGG T8: 20 booking (3 huỷ + 4 no-show), 13 hoá đơn. Hoa hồng 18.000đ/booking: 20 booking × 18.000đ = 360.000đ.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>cid</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>campaign</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>partner</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>brand</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>expire</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>kind</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>store</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>issued</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>used</t>
+        </is>
+      </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>locked</t>
+        </is>
+      </c>
+      <c r="L1" s="5" t="inlineStr">
+        <is>
+          <t>gross</t>
+        </is>
+      </c>
+      <c r="M1" s="5" t="inlineStr">
+        <is>
+          <t>disc</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>337795</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>337795 - Noire - Techcombank Reward × OneU</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>NCB</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PHAT</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>3000</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>337795</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>337795 - Noire - Techcombank Reward × OneU</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>NCB</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>DUNG</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>NCB_MET</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
+        <v>2</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>346000</v>
+      </c>
+      <c r="M3" t="n">
+        <v>51900</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>337795</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>337795 - Noire - Techcombank Reward × OneU</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>NCB</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>DUNG</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>NCB_SKC</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>593000</v>
+      </c>
+      <c r="M4" t="n">
+        <v>88950</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>337795</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>337795 - Noire - Techcombank Reward × OneU</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>NCB</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>DUNG</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>NCB_ET</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>2</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>2458000</v>
+      </c>
+      <c r="M5" t="n">
+        <v>145900</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>337795</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>337795 - Noire - Techcombank Reward × OneU</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>NCB</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>DUNG</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>NCB_MET</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
+        <v>197000</v>
+      </c>
+      <c r="M6" t="n">
+        <v>29550</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>337795</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>337795 - Noire - Techcombank Reward × OneU</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>NCB</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>DUNG</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>NCB_SKC</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="n">
+        <v>6</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>7104000</v>
+      </c>
+      <c r="M7" t="n">
+        <v>453400</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>337795</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>337795 - Noire - Techcombank Reward × OneU</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>NCB</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>DUNG</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>NCB_SKC</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" t="n">
+        <v>3</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
+        <v>1196000</v>
+      </c>
+      <c r="M8" t="n">
+        <v>179400</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>344574</t>
+        </is>
+      </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>P02</t>
+          <t>344574 - Dining - Techcombank Reward × OneU</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Cơ sở</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>NDC</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>PHAT</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>1500</v>
+      </c>
+      <c r="J9" t="n">
         <v>0</v>
       </c>
-      <c r="F9" t="n">
-        <v>2902750</v>
-      </c>
-      <c r="H9" t="n">
-        <v>17416500</v>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>344574</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>344574 - Dining - Techcombank Reward × OneU</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>NDC</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>DUNG</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
           <t>2026-09</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>P02</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Cơ sở</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>NDC_BKL</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
         <v>0</v>
       </c>
-      <c r="F10" t="n">
-        <v>2902750</v>
-      </c>
-      <c r="H10" t="n">
-        <v>20319250</v>
+      <c r="J10" t="n">
+        <v>7</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="n">
+        <v>8108000</v>
+      </c>
+      <c r="M10" t="n">
+        <v>1400000</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10</t>
+          <t>344574</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>P02</t>
+          <t>344574 - Dining - Techcombank Reward × OneU</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Cơ sở</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>NDC</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>DUNG</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>NDC_NTMK</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
         <v>0</v>
       </c>
-      <c r="F11" t="n">
-        <v>2902750</v>
-      </c>
-      <c r="H11" t="n">
-        <v>20319250</v>
+      <c r="J11" t="n">
+        <v>3</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="n">
+        <v>2550000</v>
+      </c>
+      <c r="M11" t="n">
+        <v>600000</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-11</t>
+          <t>344575</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>P02</t>
+          <t>344575 - JFB - Techcombank Reward × OneU</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Cơ sở</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>NJFB</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>PHAT</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>1500</v>
+      </c>
+      <c r="J12" t="n">
         <v>0</v>
       </c>
-      <c r="F12" t="n">
-        <v>2902750</v>
-      </c>
-      <c r="H12" t="n">
-        <v>23222000</v>
+      <c r="K12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-12</t>
+          <t>344575</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>P02</t>
+          <t>344575 - JFB - Techcombank Reward × OneU</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Cơ sở</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>NJFB</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>DUNG</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>NJFB_CRE</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
         <v>0</v>
       </c>
-      <c r="F13" t="n">
-        <v>2902750</v>
-      </c>
-      <c r="H13" t="n">
-        <v>26124750</v>
+      <c r="J13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" t="n">
+        <v>1861000</v>
+      </c>
+      <c r="M13" t="n">
+        <v>400000</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-07</t>
+          <t>344575</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>P04</t>
+          <t>344575 - JFB - Techcombank Reward × OneU</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Cơ sở</t>
-        </is>
-      </c>
-      <c r="D14" t="n">
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>NJFB</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>DUNG</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>NJFB_SSV</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
         <v>0</v>
       </c>
-      <c r="F14" t="n">
-        <v>689989</v>
-      </c>
-      <c r="G14" t="n">
-        <v>2069967</v>
-      </c>
-      <c r="H14" t="n">
-        <v>13799780</v>
-      </c>
-      <c r="I14" t="n">
-        <v>7313883.333333333</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2026-08</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>P04</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Cơ sở</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
+      <c r="J14" t="n">
+        <v>4</v>
+      </c>
+      <c r="K14" t="n">
         <v>0</v>
       </c>
-      <c r="F15" t="n">
-        <v>689989</v>
-      </c>
-      <c r="G15" t="n">
-        <v>2069967</v>
-      </c>
-      <c r="H15" t="n">
-        <v>13799780</v>
-      </c>
-      <c r="I15" t="n">
-        <v>7313883.333333333</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>2026-09</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>P04</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Cơ sở</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" t="n">
-        <v>689989</v>
-      </c>
-      <c r="G16" t="n">
-        <v>2069967</v>
-      </c>
-      <c r="H16" t="n">
-        <v>13799780</v>
-      </c>
-      <c r="I16" t="n">
-        <v>7313883.333333333</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>2026-10</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>P04</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Cơ sở</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" t="n">
-        <v>689989</v>
-      </c>
-      <c r="G17" t="n">
-        <v>2069967</v>
-      </c>
-      <c r="H17" t="n">
-        <v>13799780</v>
-      </c>
-      <c r="I17" t="n">
-        <v>7313883.333333333</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>2026-11</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>P04</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Cơ sở</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
-        <v>0</v>
-      </c>
-      <c r="F18" t="n">
-        <v>689989</v>
-      </c>
-      <c r="G18" t="n">
-        <v>2069967</v>
-      </c>
-      <c r="H18" t="n">
-        <v>13799780</v>
-      </c>
-      <c r="I18" t="n">
-        <v>7313883.333333333</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>2026-12</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>P04</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Cơ sở</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" t="n">
-        <v>689989</v>
-      </c>
-      <c r="G19" t="n">
-        <v>2069967</v>
-      </c>
-      <c r="H19" t="n">
-        <v>13799780</v>
-      </c>
-      <c r="I19" t="n">
-        <v>7313883.333333333</v>
+      <c r="L14" t="n">
+        <v>12717000</v>
+      </c>
+      <c r="M14" t="n">
+        <v>1600000</v>
       </c>
     </row>
   </sheetData>
@@ -4978,7 +6364,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:U10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5034,20 +6420,55 @@
       </c>
       <c r="K1" s="5" t="inlineStr">
         <is>
+          <t>fee</t>
+        </is>
+      </c>
+      <c r="L1" s="5" t="inlineStr">
+        <is>
+          <t>fee_period</t>
+        </is>
+      </c>
+      <c r="M1" s="5" t="inlineStr">
+        <is>
+          <t>commission_pct</t>
+        </is>
+      </c>
+      <c r="N1" s="5" t="inlineStr">
+        <is>
           <t>fee_month</t>
         </is>
       </c>
-      <c r="L1" s="5" t="inlineStr">
-        <is>
-          <t>commission_pct</t>
-        </is>
-      </c>
-      <c r="M1" s="5" t="inlineStr">
+      <c r="O1" s="5" t="inlineStr">
+        <is>
+          <t>fee_unit</t>
+        </is>
+      </c>
+      <c r="P1" s="5" t="inlineStr">
+        <is>
+          <t>fee_unit_amount</t>
+        </is>
+      </c>
+      <c r="Q1" s="5" t="inlineStr">
+        <is>
+          <t>sponsor</t>
+        </is>
+      </c>
+      <c r="R1" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="S1" s="5" t="inlineStr">
         <is>
           <t>media</t>
         </is>
       </c>
-      <c r="N1" s="5" t="inlineStr">
+      <c r="T1" s="5" t="inlineStr">
+        <is>
+          <t>owner</t>
+        </is>
+      </c>
+      <c r="U1" s="5" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -5076,7 +6497,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>NCB</t>
+          <t>NCB, NDC, NJFB</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -5091,7 +6512,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -5105,37 +6526,47 @@
       <c r="K2" t="n">
         <v>0</v>
       </c>
-      <c r="L2" t="n">
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="M2" t="n">
         <v>0</v>
       </c>
-      <c r="M2" t="n">
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>POS</t>
+        </is>
+      </c>
+      <c r="S2" t="n">
         <v>400000000</v>
       </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>3.000 mã phát 1 lô 21/07</t>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>3 chương trình mã theo brand (xem 3_CHUONG_TRINH). Kỳ HĐ lấy theo hạn mã dài nhất trên log eVoucher.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>P02</t>
+          <t>P04</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>DiningCity</t>
+          <t>HDBank Priority</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AGGREGATOR</t>
+          <t>PARTNER</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Nền tảng đặt bàn</t>
+          <t>Ngân hàng</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -5169,42 +6600,52 @@
       <c r="K3" t="n">
         <v>0</v>
       </c>
-      <c r="L3" t="n">
-        <v>0.1</v>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
       </c>
       <c r="M3" t="n">
         <v>0</v>
       </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>Phí chỗ ngồi 18k/khách + HH set menu 10%</t>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>POS</t>
+        </is>
+      </c>
+      <c r="S3" t="n">
+        <v>0</v>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>~20 bill/tháng theo kế hoạch</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>P03</t>
+          <t>P05</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Grab Dine Out</t>
+          <t>Shinhan Bank / Shinhan Finance</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AGGREGATOR</t>
+          <t>PARTNER</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Nền tảng</t>
+          <t>Ngân hàng</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>NDC, NJFB</t>
+          <t>TẤT CẢ</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -5214,17 +6655,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Chuẩn bị</t>
+          <t>Đang chạy</t>
         </is>
       </c>
       <c r="J4" t="n">
@@ -5233,27 +6669,37 @@
       <c r="K4" t="n">
         <v>0</v>
       </c>
-      <c r="L4" t="n">
-        <v>0.138</v>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
       </c>
       <c r="M4" t="n">
-        <v>172944323</v>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>Voucher giảm ngay 20% KH mới · 15% KH cũ · voucher 500k bán 375k — NOIRE fund, CMS 13,8% (báo cáo Promotion-AGG T8/2026)</t>
+        <v>0</v>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>POS</t>
+        </is>
+      </c>
+      <c r="S4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>Không phát mã — khách quẹt thẻ Shinhan tại quầy</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>P04</t>
+          <t>P06</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>HDBank Priority</t>
+          <t>Urbox</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -5263,61 +6709,42 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Ngân hàng</t>
+          <t>Ví · e-voucher</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>NDC</t>
+          <t>TẤT CẢ</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
           <t>TẤT CẢ</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>2026-12-31</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Chuẩn bị</t>
         </is>
       </c>
       <c r="J5" t="n">
         <v>1</v>
       </c>
-      <c r="K5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>Giảm 15% tổng bill, ~20 bill/tháng</t>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>POS</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Bổ sung kỳ hợp đồng, cơ chế, phí</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>P05</t>
+          <t>P07</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Shinhan Bank / Shinhan Finance</t>
+          <t>Betakee</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -5327,7 +6754,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Ngân hàng</t>
+          <t>Ví · e-voucher</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -5338,45 +6765,31 @@
       <c r="F6" t="inlineStr">
         <is>
           <t>TẤT CẢ</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Đang chạy</t>
         </is>
       </c>
       <c r="J6" t="n">
         <v>1</v>
       </c>
-      <c r="K6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" t="n">
-        <v>0</v>
-      </c>
-      <c r="M6" t="n">
-        <v>0</v>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>Mode B — không phát mã, quẹt thẻ tại quầy</t>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>POS</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>Bổ sung kỳ hợp đồng, cơ chế, phí</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>P06</t>
+          <t>P08</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Urbox</t>
+          <t>Visa</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -5386,7 +6799,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Ví · e-voucher</t>
+          <t>Tổ chức thẻ</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -5402,128 +6815,174 @@
       <c r="J7" t="n">
         <v>1</v>
       </c>
-      <c r="K7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>Chưa thấy trên POS T1–T9/2026 — bổ sung kỳ hợp đồng, cơ chế</t>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>POS</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>Chỉ tính CTKM mang tên Visa — PTTT VISA là cách khách trả tiền, không phải chương trình đối tác</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>P07</t>
+          <t>P03</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Betakee</t>
+          <t>Grab Dine Out</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>PARTNER</t>
+          <t>AGGREGATOR</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Ví · e-voucher</t>
+          <t>Dine-out · ưu đãi tại quán</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
+          <t>NDC, NJFB</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
           <t>TẤT CẢ</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>TẤT CẢ</t>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Đang chạy</t>
         </is>
       </c>
       <c r="J8" t="n">
         <v>1</v>
       </c>
-      <c r="K8" t="n">
+      <c r="M8" t="n">
+        <v>0.138</v>
+      </c>
+      <c r="N8" t="n">
         <v>0</v>
       </c>
-      <c r="L8" t="n">
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="P8" t="n">
         <v>0</v>
       </c>
-      <c r="M8" t="n">
-        <v>0</v>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>Chưa thấy trên POS T1–T9/2026 — bổ sung kỳ hợp đồng, cơ chế</t>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>NOIRE</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>POS</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>CMS 13,8% (báo cáo Promotion-AGG T8/2026). Hoá đơn nhận theo cột Nguồn = GRABFOOD trên POS.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>P08</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Visa</t>
+          <t>GrabFood (giao hàng)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>PARTNER</t>
+          <t>AGGREGATOR</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Tổ chức thẻ</t>
+          <t>Giao hàng</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
+          <t>NCB</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
           <t>TẤT CẢ</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>TẤT CẢ</t>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Đang chạy</t>
         </is>
       </c>
       <c r="J9" t="n">
         <v>1</v>
       </c>
-      <c r="K9" t="n">
+      <c r="M9" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="N9" t="n">
         <v>0</v>
       </c>
-      <c r="L9" t="n">
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="P9" t="n">
         <v>0</v>
       </c>
-      <c r="M9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>Chỉ tính CTKM mang tên Visa — PTTT VISA là cách khách trả tiền, không phải chương trình đối tác</t>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>NOIRE</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>POS</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>Hoa hồng ghi ngay trên hoá đơn POS (≈25%).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>P11</t>
+          <t>P02</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>GrabFood (giao hàng)</t>
+          <t>Dining City</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -5533,17 +6992,27 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Nền tảng giao hàng</t>
+          <t>Đặt bàn</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>NCB</t>
+          <t>NDC, NJFB</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
           <t>TẤT CẢ</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -5554,18 +7023,33 @@
       <c r="J10" t="n">
         <v>1</v>
       </c>
-      <c r="K10" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" t="n">
-        <v>0.25</v>
-      </c>
       <c r="M10" t="n">
         <v>0</v>
       </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>Hoa hồng ghi ngay trên hoá đơn POS (≈25%)</t>
+      <c r="N10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Theo booking</t>
+        </is>
+      </c>
+      <c r="P10" t="n">
+        <v>18000</v>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>NOIRE</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>TU_THONG_KE</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>POS KHÔNG ghi nhận được Dining City — nhập số ở file Aggregator theo tháng (03_Aggregator · AGG_THANG). Hoa hồng 18.000đ/booking.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: so lieu T9.2026 du 30 ngay + target Q4.2026
- Tracking Sales dựng lại từ revenue-report-group-by-date T1-T9.2026 (01/01 → 30/09)
- POS T9: bảng kê hoá đơn + báo cáo bán hàng đủ tháng (hai file bị đặt nhầm tên, đã đổi lại)
- 01_master.dim_target: thêm T10–T12 cho 7 cửa hàng chính từ config_targets.csv
- tools/tracking.py: thêm đường dẫn mới của build_tracking.py (1. FnB/09 Tracking Sales Tool)
- Chốt QA 16/17 (chỉ #8 độ phủ COGS còn đỏ) · rollup khớp báo cáo tháng 84/84

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data_input/01_master.xlsx
+++ b/data_input/01_master.xlsx
@@ -1,32 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="_HƯỚNG DẪN" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="dim_store" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="dim_target" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="dim_cogs" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="budget_brand" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="budget_extra" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="budget_channel" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="budget_store" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="partners" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="pre_analytics" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="crm_target" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="system_tools" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="system_dashboards" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="system_caches" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="_stats" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="partner_plan" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="partner_program" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="partner_agg" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="partner_voucher" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="partner_ingest" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_HƯỚNG DẪN" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="dim_store" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="dim_target" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="dim_cogs" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="budget_brand" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="budget_extra" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="budget_channel" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="budget_store" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="partners" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pre_analytics" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="crm_target" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_tools" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_dashboards" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_caches" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_stats" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="partner_plan" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="partner_program" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="partner_agg" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="partner_voucher" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="partner_ingest" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -5103,7 +5103,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -5576,6 +5576,321 @@
       </c>
       <c r="C31" t="n">
         <v>346823618</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>NCB_ET</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>1111585212</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>NCB_MET</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>1033665321</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>NCB_SKC</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>726439552</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>NDC_BKL</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>1020922867</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>NDC_NTMK</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>1631650939</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>NJFB_CRE</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>1794816033</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>NJFB_SSV</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>879728850</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-11</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>NCB_ET</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>1107999453</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-11</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>NCB_MET</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>1030330917</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-11</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>NCB_SKC</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>738156319</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-11</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>NDC_BKL</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>1057149162</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-11</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>NDC_NTMK</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>1657967889</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-11</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>NJFB_CRE</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>1823764678</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-11</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>NJFB_SSV</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>936485550</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-12</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>NCB_ET</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>1262288377</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-12</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>NCB_MET</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>1151446317</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-12</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>NCB_SKC</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>840944586</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-12</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>NDC_BKL</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>1261707525</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-12</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>NDC_NTMK</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>1888839918</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-12</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>NJFB_CRE</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>2073012518</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-12</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>NJFB_SSV</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>1168499845</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data(m9): nap T9 - lay PTTT GRAB DEBIT lam can cu du lieu Grab + hoa hong/uu dai Grab T9 thuc
- data_contract.json $partner.pos: them co pttt_confirmed (HD tra GRAB DEBIT, ke ca Nguon TAI CHO, tinh cho Grab; bo co = quay lai XAC_NHAN)
- tools/monthly_lib.py partner_of_bill doc co moi (them tuy chon, mac dinh giu hanh vi cu)
- T9: Doi tac 246,4 tr (Aggregator 205,4 tr / Partner 41,0 tr), M7 = M9; Grab Dine Out 154 HD khop bao cao team 156 don
- Dining City T9 (13 HD, 12,6 tr, hoa hong 252k), eVoucher Techcombank log tem 30/09
- docs/modules/M9_Partnership.md cap nhat quy tac + so lieu

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data_input/01_master.xlsx
+++ b/data_input/01_master.xlsx
@@ -3474,7 +3474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P5"/>
+  <dimension ref="A1:O6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3553,11 +3553,6 @@
           <t>note</t>
         </is>
       </c>
-      <c r="P1" s="5" t="inlineStr">
-        <is>
-          <t>_src</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3646,7 +3641,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-09</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -3654,71 +3649,97 @@
           <t>NDC</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>NDC_NTMK</t>
-        </is>
-      </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>P03</t>
-        </is>
-      </c>
-      <c r="G4" t="n">
-        <v>96</v>
+          <t>P02</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>14</v>
       </c>
       <c r="H4" t="n">
-        <v>41</v>
-      </c>
-      <c r="J4" t="n">
-        <v>1570000</v>
+        <v>13</v>
+      </c>
+      <c r="I4" t="n">
+        <v>12597000</v>
+      </c>
+      <c r="L4" t="n">
+        <v>252000</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>18.000đ/booking</t>
+        </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>nguồn: NOIRE_Bao_Cao_Promotion AGG - MKT_T8-2026.xlsx · C2 · báo cáo ghi Sales 31.176.000 (trước VAT)</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>raw</t>
+          <t>Báo cáo Aggregator T9 (Theo_Thang 9): 13 hoá đơn, DT 12.597.000, hoa hồng 252.000đ = 14 booking × 18.000đ (số booking suy từ hoa hồng; huỷ/no-show, khách đến chưa có).</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-09</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>NDC</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>P03</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>14666565</v>
+      </c>
+      <c r="L5" t="n">
+        <v>8446135</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Sao kê/báo cáo team T9</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Báo cáo Aggregator T9: discount 37.623.816 (NOIRE fund) · hoa hồng 21.666.685 cho 156 đơn Grab (POS: 154 HĐ GRAB DEBIT). Chia theo doanh thu POS: NDC 39.0%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
           <t>NJFB</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>NJFB_CRE</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>P03</t>
         </is>
       </c>
-      <c r="G5" t="n">
-        <v>76</v>
-      </c>
-      <c r="H5" t="n">
-        <v>29</v>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>nguồn: NOIRE_Bao_Cao_Promotion AGG - MKT_T8-2026.xlsx · C2 · báo cáo ghi Sales 49.942.000 (trước VAT)</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>raw</t>
+      <c r="J6" t="n">
+        <v>22957251</v>
+      </c>
+      <c r="L6" t="n">
+        <v>13220550</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Sao kê/báo cáo team T9</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Báo cáo Aggregator T9: discount 37.623.816 (NOIRE fund) · hoa hồng 21.666.685 cho 156 đơn Grab (POS: 154 HĐ GRAB DEBIT). Chia theo doanh thu POS: NJFB 61.0%.</t>
         </is>
       </c>
     </row>
@@ -3733,7 +3754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M14"/>
+  <dimension ref="A1:M15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4178,34 +4199,34 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>NCB_SKC</t>
+          <t>NCB_MET</t>
         </is>
       </c>
       <c r="I8" t="n">
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K8" t="n">
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>1196000</v>
+        <v>344000</v>
       </c>
       <c r="M8" t="n">
-        <v>179400</v>
+        <v>51600</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>344574</t>
+          <t>337795</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>344574 - Dining - Techcombank Reward × OneU</t>
+          <t>337795 - Noire - Techcombank Reward × OneU</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -4215,38 +4236,43 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>NDC</t>
+          <t>NCB</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-10-31</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>PHAT</t>
+          <t>DUNG</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>NCB_SKC</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="K9" t="n">
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>0</v>
+        <v>1561000</v>
       </c>
       <c r="M9" t="n">
-        <v>0</v>
+        <v>234150</v>
       </c>
     </row>
     <row r="10">
@@ -4277,33 +4303,28 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>DUNG</t>
+          <t>PHAT</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-09</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>NDC_BKL</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
       <c r="J10" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="K10" t="n">
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>8108000</v>
+        <v>0</v>
       </c>
       <c r="M10" t="n">
-        <v>1400000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -4344,34 +4365,34 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>NDC_NTMK</t>
+          <t>NDC_BKL</t>
         </is>
       </c>
       <c r="I11" t="n">
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="K11" t="n">
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>2550000</v>
+        <v>11468000</v>
       </c>
       <c r="M11" t="n">
-        <v>600000</v>
+        <v>2000000</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>344575</t>
+          <t>344574</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>344575 - JFB - Techcombank Reward × OneU</t>
+          <t>344574 - Dining - Techcombank Reward × OneU</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -4381,7 +4402,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>NJFB</t>
+          <t>NDC</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -4391,28 +4412,33 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>PHAT</t>
+          <t>DUNG</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>NDC_NTMK</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="K12" t="n">
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>0</v>
+        <v>4670000</v>
       </c>
       <c r="M12" t="n">
-        <v>0</v>
+        <v>1200000</v>
       </c>
     </row>
     <row r="13">
@@ -4443,33 +4469,28 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>DUNG</t>
+          <t>PHAT</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-09</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>NJFB_CRE</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
       <c r="J13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" t="n">
         <v>1</v>
       </c>
-      <c r="K13" t="n">
-        <v>0</v>
-      </c>
       <c r="L13" t="n">
-        <v>1861000</v>
+        <v>0</v>
       </c>
       <c r="M13" t="n">
-        <v>400000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -4510,23 +4531,80 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
+          <t>NJFB_CRE</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" t="n">
+        <v>3</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" t="n">
+        <v>5843000</v>
+      </c>
+      <c r="M14" t="n">
+        <v>1200000</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>344575</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>344575 - JFB - Techcombank Reward × OneU</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>NJFB</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>DUNG</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
           <t>NJFB_SSV</t>
         </is>
       </c>
-      <c r="I14" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" t="n">
-        <v>4</v>
-      </c>
-      <c r="K14" t="n">
-        <v>0</v>
-      </c>
-      <c r="L14" t="n">
-        <v>12717000</v>
-      </c>
-      <c r="M14" t="n">
-        <v>1600000</v>
+      <c r="I15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" t="n">
+        <v>7</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" t="n">
+        <v>19862000</v>
+      </c>
+      <c r="M15" t="n">
+        <v>2800000</v>
       </c>
     </row>
   </sheetData>
@@ -4987,7 +5065,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5054,41 +5132,6 @@
       <c r="F2" t="inlineStr">
         <is>
           <t>danh mục: điền 12 ô còn trống: P02·media, P03·media, P06·commission_pct, P06·media, P06·fee, P07·commission_pct … · chương trình: điền 11 ô còn trống: P02-CU1·rate, P02-CU1·cap, P02-CU1·min_bill, P03-CU1·cap, P03-CU1·min_bill, P04-CU1·cap …</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>S19_aggregator</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>NOIRE_Bao_Cao_Promotion AGG - MKT_T8-2026.xlsx</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>bao_cao_agg</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Báo cáo Promotion-AGG của team (sheet Aggregator · mục C2) → agg 2 dòng</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>số aggregator: thêm 2 dòng chưa có ở file chuẩn: 2026-08/P03/NDC/NDC_NTMK, 2026-08/P03/NJFB/NJFB_CRE</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>2026-08 · NDC_NTMK: Doanh thu để trống — báo cáo ghi Sales trước VAT, cần Tổng tiền hoá đơn (gồm VAT &amp; phí phục vụ) · 2026-08 · NJFB_CRE: Doanh thu để trống — báo cáo ghi Sales trước VAT, cần Tổng tiền hoá đơn (gồm VAT &amp; phí phục vụ) · 2026-08: dòng 'Dingning City' chưa nhận ra — khai tên này vào cột 'Tên khác trên báo cáo' của 2_AGGREGATOR (hoặc bí danh cửa hàng ở dim_store)</t>
         </is>
       </c>
     </row>

</xml_diff>